<commit_message>
chore(editais): atualizacao automatica 2026-09-14 13:50
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1012,46 +1020,118 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Novo - e-mail enviado em 14/09/2026</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
+          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 200.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
+2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
+2026-10-23 a 2026-10-29: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
+2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
           <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
 2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
@@ -1072,70 +1152,70 @@
 2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O edital visa incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCC) com foco em inovação, empreendedorismo e aplicabilidade prática. Serão concedidas Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para propostas que apresentem soluções inovadoras e empreendedoras, com impacto econômico, social e/ou ambiental no Espírito Santo, alinhadas aos ODS da ONU (especialmente 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Podem submeter propostas professores orientadores com vínculo estatutário ou celetista por tempo indeterminado a IES reconhecidas pelo MEC e localizadas no Espírito Santo, que não estejam afastados da IES, estejam adimplentes com a FAPES, residam no ES ou municípios limítrofes, e possuam currículo Lattes atualizado. Cada proponente deve submeter entre 3 e 5 propostas, cada uma vinculada a um único aluno. Se os alunos orientados estiverem vinculados a outra IES, o proponente deve apresentar declaração de autorização de ambas as IES. Os alunos orientados devem ser estudantes regulares de graduação em IES localizadas no Espírito Santo, com desempenho acadêmico igual ou superior a 7.0, adimplentes com a FAPES, com o proponente como professor orientador durante todo o período da bolsa, residência no ES ou municípios limítrofes, e cadastrados no Sigfapes. As IES devem ser públicas ou privadas, localizadas no ES, e prestar anuência às propostas.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até as 17h59)
 ?: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção)
@@ -1148,70 +1228,70 @@
 ?: Prazo de contratação (Terceira Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital aceita todos os formatos de TCC definido pelas DCNs, como monografia, dissertação, projeto experimental, relatório técnico ou científico, artigo, plano de negócios e outros. As propostas concorrerão com as demais de suas respectivas microrregiões. Serão apoiados no máximo 20 projetos de TCC por microrregião na primeira chamada, e até 10 projetos de TCC por microrregião nas segunda e terceira chamadas. Recursos financeiros remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Propostas com Nota Final (NF) inferior a 70 pontos serão desclassificadas. Em caso de empate na NF, serão utilizados os critérios de avaliação 1, 2, 3, 4 e 5, nesta ordem, para desempate. Persistindo o empate, será selecionada a proposta submetida primeiro. Não é permitido o acúmulo de bolsas FAPES com outras bolsas, exceto as do Programa Nossa Bolsa, Programa Universidade para Todos (Prouni) e Bolsas de Extensão (Ext-E e Ext-F). O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes (https://fapes.es.gov.br/valores-de-bolsas-e-auxilios) na data de publicação deste edital. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. O orientador receberá até dois auxílios para orientação de TCC: o primeiro após a contratação e o segundo quando pelo menos um aluno orientado apresentar a Ata de Defesa do TCC. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1221,157 +1301,89 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)
 ?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação e análise de mérito)
 2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
         <is>
           <t>Os valores por proposta variam conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é baseada nas seguintes pontuações: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos) e Nível Básico (60 a 75 pontos). Os recursos financeiros remanescentes serão redirecionados para propostas suplentes nos níveis de maturidade I, II e III, nesta ordem, respeitando a classificação. O projeto terá prazo de vigência de 24 meses, sem prorrogação. Mínimo de 20% do valor total solicitado deve ser destinado a bolsas. Parte dos recursos de custeio deve ser destinada à associação à Anprotec. Serão permitidas exclusivamente bolsas na modalidade BPIG, níveis II a X, por no máximo 24 meses.</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1395,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1393,53 +1405,53 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>R$ 300.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1463,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1459,20 +1471,32 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 300.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>R$ 150.000,00</t>
+        </is>
+      </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
@@ -1480,22 +1504,22 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1531,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
+          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1519,39 +1543,39 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
+          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
         </is>
       </c>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
+          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1587,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1575,48 +1599,39 @@
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I17" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1628,7 +1643,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1640,96 +1655,161 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1741,17 +1821,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N19" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-15 12:28
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -744,7 +736,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-08-07 a 2026-09-14: Envio da proposta e documentos (via SigFapes, até as 17h59)</t>
+          <t>2026-09-25 a 2026-10-01: Prazo para recorrer (habilitação) (5 dias úteis após o resultado preliminar da habilitação)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -1023,9 +1015,9 @@
           <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Novo - e-mail enviado em 14/09/2026</t>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-16 12:22
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,12 +29,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,12 +54,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -726,7 +734,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
+          <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -736,28 +744,28 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25 a 2026-10-01: Prazo para recorrer (habilitação) (5 dias úteis após o resultado preliminar da habilitação)</t>
+          <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos visa apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. Seu objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, bem como consolidar grupos de referência em áreas do conhecimento e setores estratégicos do estado.</t>
+          <t>O Edital Fapes n° 24/2026 (PPP-ES) tem como objetivo apoiar o primeiro projeto de pesquisa científica de pesquisadores doutores em início de carreira. Ele visa promover o acesso a recursos para o desenvolvimento de seus primeiros projetos, fortalecer a infraestrutura de pesquisa e apoiar a formação e consolidação de novos grupos de pesquisa no Estado do Espírito Santo. Os projetos devem estar vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, localizadas no Espírito Santo, e contemplar as 8 grandes áreas do conhecimento do CNPq, com duração de até 24 meses.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas. A equipe executora deve ser exclusiva e composta por no mínimo 7 pesquisadores doutores, além do coordenador, com representação da Instituição Executora, outras IES/P capixabas, IES/P de fora do estado ou do País, e um pesquisador vinculado a órgão ou instituição pública estadual.</t>
+          <t>Pesquisadores doutores em início de carreira, com título obtido a partir de 28/08/2018, que possuam vínculo estatutário ou celetista por tempo indeterminado com uma Instituição de Ensino Superior e/ou de Pesquisa (IES/P) pública ou privada localizada no Espírito Santo, residam no Espírito Santo ou em município limítrofe, e que não tenham atuado como coordenador de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq (com exceções específicas).</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>R$ 12.000.000,00</t>
+          <t>R$ 4.000.000,00</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>R$ 1.200.000,00</t>
+          <t>R$ 180.000,00</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
@@ -766,77 +774,6 @@
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-07 a 2026-09-14: Envio da proposta e documentos (via SigFapes, até as 17h59)
-2026-09-10: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
-2026-09-25 a 2026-10-01: Prazo para recorrer (habilitação) (5 dias úteis após o resultado preliminar da habilitação)
-2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após o resultado preliminar de análise de mérito)</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>A Fapes pode alterar as datas e os prazos do cronograma por necessidade administrativa ou decisão institucional. Cada coordenador pode apresentar apenas uma proposta, sendo a última enviada considerada válida em caso de múltiplas submissões. A etapa de habilitação é eliminatória. Serão classificadas apenas as propostas com nota final igual ou superior a 70,0 pontos. Em caso de empate na nota final, o desempate será pela maior nota nos critérios de avaliação (item 3.2.1) na ordem apresentada, e persistindo o empate, pela proposta submetida primeiro. A proposta aprovada não poderá ser alterada no momento da contratação. O projeto aprovado não será contratado se o coordenador não cumprir as condições, apresentar informações falsas ou não atender aos requisitos, resultando na convocação de suplentes. A Fapes não reivindicará direitos de participação na propriedade intelectual sobre as pesquisas e projetos apoiados. É obrigatória a menção clara e destacada do apoio da Fapes em todas as publicações e divulgações relacionadas ao projeto.</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_21-2026_-_Redes_de_PDI_em_Setores_Estratégicos.pdf</t>
-        </is>
-      </c>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>pesquisa/EDITAL_FAPES_No_21_2026_-_REDES_DE_PESQUISA,_DESENVOLVIMENTO_E_INOVAÇÃO_EM_SETORES_ESTRATÉGICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisa</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>O Edital Fapes n° 24/2026 (PPP-ES) tem como objetivo apoiar o primeiro projeto de pesquisa científica de pesquisadores doutores em início de carreira. Ele visa promover o acesso a recursos para o desenvolvimento de seus primeiros projetos, fortalecer a infraestrutura de pesquisa e apoiar a formação e consolidação de novos grupos de pesquisa no Estado do Espírito Santo. Os projetos devem estar vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, localizadas no Espírito Santo, e contemplar as 8 grandes áreas do conhecimento do CNPq, com duração de até 24 meses.</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores doutores em início de carreira, com título obtido a partir de 28/08/2018, que possuam vínculo estatutário ou celetista por tempo indeterminado com uma Instituição de Ensino Superior e/ou de Pesquisa (IES/P) pública ou privada localizada no Espírito Santo, residam no Espírito Santo ou em município limítrofe, e que não tenham atuado como coordenador de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq (com exceções específicas).</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 4.000.000,00</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>R$ 180.000,00</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
 2026-08-29 a 2026-09-30: Envio da proposta e documentos (até as 17h59, via SigFapes)
@@ -845,19 +782,96 @@
 2026-12-10: Envio de documentos para contratação (O coordenador receberá informações com prazo e documentação necessária via SigFapes.)</t>
         </is>
       </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Projetos aprovados terão duração máxima de 24 meses e devem estar enquadrados em uma das 8 grandes áreas do conhecimento do CNPq. A Fapes reserva-se o direito de alterar as datas e prazos do cronograma por necessidade administrativa ou decisão institucional. É fundamental que o coordenador mantenha seus dados cadastrais atualizados no sistema SigFapes para garantir o recebimento das comunicações oficiais. A proposta aprovada não poderá ser alterada no momento da contratação, e a ausência da documentação ética e legal exigida impedirá a contratação do projeto.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2024-2026%20PPP-ES.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>pesquisa/EDITAL_FAPES_No_24_2026_-_PRIMEIROS_PROJETOS_DE_PESQUISA_-_ESPÍRITO_SANTO_(PPP-ES).pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 16/09/2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (Até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 28/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado." → "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Os objetivos específicos incluem valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, ampliar a divulgação da ciência e fortalecer a visibilidade institucional da Fundação."
+Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também se destina a profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação."
+Valor por proposta: "R$ 12.000,00" → "R$ 12.000,00 (1º lugar); R$ 8.000,00 (menção honrosa)"</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Os objetivos específicos incluem valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, ampliar a divulgação da ciência e fortalecer a visibilidade institucional da Fundação.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também se destina a profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 308.000,00</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000,00 (1º lugar); R$ 8.000,00 (menção honrosa)</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (Até 17h59)
+2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (Até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 28/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
+?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)
+2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo (Votação entre as 3 matérias mais bem classificadas em cada subcategoria.)</t>
+        </is>
+      </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Projetos aprovados terão duração máxima de 24 meses e devem estar enquadrados em uma das 8 grandes áreas do conhecimento do CNPq. A Fapes reserva-se o direito de alterar as datas e prazos do cronograma por necessidade administrativa ou decisão institucional. É fundamental que o coordenador mantenha seus dados cadastrais atualizados no sistema SigFapes para garantir o recebimento das comunicações oficiais. A proposta aprovada não poderá ser alterada no momento da contratação, e a ausência da documentação ética e legal exigida impedirá a contratação do projeto.</t>
+          <t>Esta edição do Prêmio Fapes homenageia a Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. A premiação possui caráter exclusivamente honorífico, meritório e eventual, não configurando contraprestação por serviços prestados, vínculo empregatício, relação de trabalho, bolsa de pesquisa ou remuneração continuada. É permitida apenas uma inscrição por pessoa neste edital, sendo a última enviada considerada válida em caso de múltiplas submissões. A Fapes garante condições de acessibilidade às pessoas com deficiência durante o processo de inscrição. O participante autoriza o uso de seu nome, imagem, voz e demais informações para fins institucionais e de divulgação do prêmio, sem remuneração. O tratamento dos dados pessoais seguirá a Lei Federal nº 13.709/2018 (LGPD).</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2024-2026%20PPP-ES.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>pesquisa/EDITAL_FAPES_No_24_2026_-_PRIMEIROS_PROJETOS_DE_PESQUISA_-_ESPÍRITO_SANTO_(PPP-ES).pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -869,7 +883,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
+          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -879,28 +893,28 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)</t>
+          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado.</t>
+          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados.</t>
+          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>R$ 308.000,00</t>
+          <t>R$ 3.000.000,00</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>R$ 12.000,00</t>
+          <t>R$ 200.000,00</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
@@ -909,149 +923,6 @@
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (até 17h59)
-2026-06-22 a 2026-09-15: Envio das inscrições – Categoria Jornalismo (até 17h59)
-?: Prazo para recurso administrativo (5 (cinco) dias úteis após a divulgação do resultado preliminar)</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Esta edição do edital é em homenagem à Professora Jurema José de Oliveira. Para as categorias Projetos e Destaque, as 3 (três) propostas com as maiores notas seguem para votação pelo Comitê de Especialistas, que votará o 1º lugar e as duas menções honrosas. Para a categoria Jornalismo, as 3 (três) matérias com maiores notas seguem para votação popular, onde a matéria com o maior número de votos será considerada vencedora, e as duas seguintes receberão menção honrosa. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. Os contemplados deverão protocolar solicitação de pagamento no prazo máximo de até 90 (noventa) dias, contados da data de publicação do resultado final no DIO-ES. Para a categoria Jornalismo, a matéria deve ter sido veiculada entre 01/09/2025 a 15/09/2026 e disponibilizada no canal oficial do veículo de comunicação.</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES N° 25/2025 - PARTICIPAÇÃO DE EQUIPES DE ESTUDANTES EM MOSTRAS E COMPETIÇÕES TÉCNICO-CIENTÍFICAS</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Conceder apoio financeiro a equipes formadas por estudantes de nível médio, de graduação e pós-graduação, coordenadas por um professor orientador. O objetivo é permitir a participação dessas equipes em mostras e competições técnico-científicas de âmbito regional, nacional ou internacional, visando a divulgação e difusão de resultados obtidos por instituições de ensino do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Professores(as) coordenadores(as) de equipes de 3 a 5 estudantes, vinculados(as) a instituições de ensino médio públicas ou instituições de ensino superior públicas ou privadas localizadas no estado do Espírito Santo. O proponente deve ter formação mínima de nível superior, vínculo ativo com a instituição, atuar em sala de aula na mesma instituição dos estudantes, ter Lattes atualizado há menos de 6 meses, estar regularizado junto à Fapes e morar no Espírito Santo ou municípios limítrofes. Estudantes de instituições privadas devem ser bolsistas integrais financiados por programas governamentais estaduais ou federais.</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>R$ 500.000,00</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br, sucon@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>?: Prazo para impugnação do edital (5 dias úteis antes do encerramento do prazo de submissão da 1ª Chamada)
-2025-11-10 a 2025-12-16: Submissão de propostas (Até as 17h:59. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 1ª Chamada (eventos com início entre 01/03/2026 a 30/06/2026))
-2026-03-04 a 2026-04-09: Submissão de propostas (Até as 17:59h. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 2ª Chamada (eventos com início entre 01/07/2026 a 31/12/2026))
-2026-08-04 a 2026-09-11: Submissão de propostas (Até as 17h:59. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
-?: Interposição de recursos administrativos (5 dias úteis a partir da publicação do resultado preliminar. Para 3ª Chamada (eventos com início entre 04/01/2027 a 30/04/2027))
-?: Contratação e assinatura do Termo de Outorga (Até 30 dias após a publicação do resultado final homologado. Período específico de assinatura será definido após a homologação.)
-?: Prazo para informar dados bancários (Até 30 dias após a assinatura e publicação do Termo de Outorga)
-?: Prazo para prestação de contas (Até 30 dias após o término da vigência do Termo de Outorga)</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>O valor por proposta varia conforme a categoria do evento: R$ 500,00 para eventos regionais, R$ 1.200,00 para eventos nacionais e US$ 1.500,00 para eventos internacionais. O edital prevê três chamadas com períodos de submissão e eventos distintos. O início do evento proposto deve corresponder ao período da chamada selecionada. A Fapes pode alterar as datas e prazos definidos no cronograma. Cada coordenador pode apresentar apenas uma proposta. Não são contempladas propostas para participação em concursos ou premiações sem natureza acadêmica, técnico-científica ou tecnológica, ou competições esportivas.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_N_25_2025_Participação_Equipe_em_Mostras_e_Competições-2.pdf</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_N°_25_2025_-_PARTICIPAÇÃO_DE_EQUIPES_DE_ESTUDANTES_EM_MOSTRAS_E_COMPETIÇÕES_TÉCNICO-CIENTÍFICAS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 200.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
 2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
@@ -1060,70 +931,70 @@
 2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
 2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
@@ -1144,70 +1015,70 @@
 2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O edital visa incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCC) com foco em inovação, empreendedorismo e aplicabilidade prática. Serão concedidas Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para propostas que apresentem soluções inovadoras e empreendedoras, com impacto econômico, social e/ou ambiental no Espírito Santo, alinhadas aos ODS da ONU (especialmente 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Podem submeter propostas professores orientadores com vínculo estatutário ou celetista por tempo indeterminado a IES reconhecidas pelo MEC e localizadas no Espírito Santo, que não estejam afastados da IES, estejam adimplentes com a FAPES, residam no ES ou municípios limítrofes, e possuam currículo Lattes atualizado. Cada proponente deve submeter entre 3 e 5 propostas, cada uma vinculada a um único aluno. Se os alunos orientados estiverem vinculados a outra IES, o proponente deve apresentar declaração de autorização de ambas as IES. Os alunos orientados devem ser estudantes regulares de graduação em IES localizadas no Espírito Santo, com desempenho acadêmico igual ou superior a 7.0, adimplentes com a FAPES, com o proponente como professor orientador durante todo o período da bolsa, residência no ES ou municípios limítrofes, e cadastrados no Sigfapes. As IES devem ser públicas ou privadas, localizadas no ES, e prestar anuência às propostas.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até as 17h59)
 ?: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção)
@@ -1220,70 +1091,70 @@
 ?: Prazo de contratação (Terceira Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O edital aceita todos os formatos de TCC definido pelas DCNs, como monografia, dissertação, projeto experimental, relatório técnico ou científico, artigo, plano de negócios e outros. As propostas concorrerão com as demais de suas respectivas microrregiões. Serão apoiados no máximo 20 projetos de TCC por microrregião na primeira chamada, e até 10 projetos de TCC por microrregião nas segunda e terceira chamadas. Recursos financeiros remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Propostas com Nota Final (NF) inferior a 70 pontos serão desclassificadas. Em caso de empate na NF, serão utilizados os critérios de avaliação 1, 2, 3, 4 e 5, nesta ordem, para desempate. Persistindo o empate, será selecionada a proposta submetida primeiro. Não é permitido o acúmulo de bolsas FAPES com outras bolsas, exceto as do Programa Nossa Bolsa, Programa Universidade para Todos (Prouni) e Bolsas de Extensão (Ext-E e Ext-F). O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes (https://fapes.es.gov.br/valores-de-bolsas-e-auxilios) na data de publicação deste edital. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. O orientador receberá até dois auxílios para orientação de TCC: o primeiro após a contratação e o segundo quando pelo menos um aluno orientado apresentar a Ata de Defesa do TCC. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1293,31 +1164,169 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Inovação</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>R$ 4.500.000,00</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>R$ 252.000,00</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>duvidas.inovacao@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)
+?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação e análise de mérito)
+2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Os valores por proposta variam conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é baseada nas seguintes pontuações: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos) e Nível Básico (60 a 75 pontos). Os recursos financeiros remanescentes serão redirecionados para propostas suplentes nos níveis de maturidade I, II e III, nesta ordem, respeitando a classificação. O projeto terá prazo de vigência de 24 meses, sem prorrogação. Mínimo de 20% do valor total solicitado deve ser destinado a bolsas. Parte dos recursos de custeio deve ser destinada à associação à Anprotec. Serão permitidas exclusivamente bolsas na modalidade BPIG, níveis II a X, por no máximo 24 meses.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA CONFAP CDTI 2026</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>€ 75.000,00</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+        </is>
+      </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Inovação</t>
+          <t>Chamadas Internacionais</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1327,55 +1336,53 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>R$ 4.500.000,00</t>
+          <t>R$ 300.000,00</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>R$ 252.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>duvidas.inovacao@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)
-?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação e análise de mérito)
-2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Os valores por proposta variam conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é baseada nas seguintes pontuações: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos) e Nível Básico (60 a 75 pontos). Os recursos financeiros remanescentes serão redirecionados para propostas suplentes nos níveis de maturidade I, II e III, nesta ordem, respeitando a classificação. O projeto terá prazo de vigência de 24 meses, sem prorrogação. Mínimo de 20% do valor total solicitado deve ser destinado a bolsas. Parte dos recursos de custeio deve ser destinada à associação à Anprotec. Serão permitidas exclusivamente bolsas na modalidade BPIG, níveis II a X, por no máximo 24 meses.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1387,7 +1394,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1395,55 +1402,52 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
+      <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>US$ 18.000,00</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>€ 75.000,00</t>
+          <t>US$ 6.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1459,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA HORIZON EUROPE</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1463,55 +1467,49 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
+      <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>R$ 300.000,00</t>
-        </is>
-      </c>
+          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
+?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
+?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1521,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; DAAD 2026</t>
+          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1531,277 +1529,38 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
+        </is>
+      </c>
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Este edital visa apoiar a manutenção de bolsas de doutorado da FAPES para bolsistas que forem aprovados na seleção do Serviço Alemão de Intercâmbio Acadêmico (DAAD). O apoio será concedido durante o período em que o bolsista realizar suas pesquisas em uma instituição na Alemanha, complementando o programa de auxílio para doutorandos brasileiros com bolsa nacional.</t>
+          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Doutorandos que forem selecionados pelo DAAD, estejam adimplentes junto à FAPES e não estejam no primeiro nem no último ano do doutorado.</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
+          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>EUR 100.000,00</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
-        <is>
-          <t>?: Submissão de propostas na Plataforma do DAAD (Para a Chamada DAAD 2026. O conteúdo completo da chamada está disponível no site do CONFAP.)</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Este documento apresenta as diretrizes específicas da FAPES para a Chamada CONFAP &amp; DAAD 2026. Para informações completas sobre a chamada, consulte o link fornecido no site do CONFAP.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20-%20FAPES%202026-1.pdf</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_DAAD_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA MOBILITY CONFAP ITALY 2026</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>As Fundações Estaduais de Amparo à Pesquisa (FAPs) brasileiras, articuladas através do CONFAP, lançam uma chamada para apoiar pesquisadores do Brasil, vinculados a instituições de ensino superior e pesquisa, que desejam desenvolver atividades de pesquisa na Itália em colaboração com colegas locais. O objetivo é facilitar e apoiar a colaboração científica, tecnológica e de inovação, promovendo a mobilidade de estudantes de doutorado, mestrado e pós-doutores, através da concessão de bolsas de estudo para fortalecer grupos de pesquisa.</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores de doutorado, mestrado e pós-doutorado vinculados a universidades e instituições de pesquisa dos Estados brasileiros participantes desta chamada (incluindo Espírito Santo - FAPES). Todos os candidatos devem ter um supervisor associado a uma universidade na Itália, parte da rede MCI. Critérios de elegibilidade adicionais podem ser definidos pelas FAPs individuais.</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-04: Prazo final para submissão de propostas (até 23:59 (horário de Brasília) via https://sistema.confap.org.br)</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Não serão cobradas taxas de matrícula por nenhuma das partes para a mobilidade de intercâmbio. Em caso de mobilidade no âmbito de projetos com potencial valor comercial e direitos de propriedade intelectual, as instituições anfitriãs e de envio devem assinar um acordo de colaboração específico. Os candidatos devem consultar suas respectivas FAPs para critérios de elegibilidade adicionais, diretrizes específicas e possíveis requisitos para submissão em suas próprias plataformas. Os documentos exigidos para as propostas de projeto incluem: proposta de projeto, Curriculum Vitae do candidato (Brasil), Curriculum Vitae do Supervisor (Itália) e carta de apoio assinada pelo supervisor (Itália).</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-MCI-–-MOBILITY-CONFAP-ITALY-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_MOBILITY_CONFAP_ITALY_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>US$ 18.000,00</t>
-        </is>
-      </c>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>US$ 6.000,00</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
-        </is>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA HORIZON EUROPE</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>€ 25.000,00 por ano de projeto</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
-?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
-?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr">
-        <is>
-          <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
-        </is>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>EUR 100.000,00</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1813,17 +1572,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N20" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-17 12:28
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -734,46 +734,122 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
+          <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Atualizado - e-mail enviado em 17/09/2026</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07 a 2026-09-21: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Objetivo: "O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos visa apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. Seu objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, bem como consolidar grupos de referência em áreas do conhecimento e setores estratégicos do estado." → "O edital visa apoiar financeiramente a criação e o fortalecimento de redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos no Espírito Santo. O objetivo é consolidar grupos de referência em áreas do conhecimento e setores estratégicos, promovendo ações coletivas de PD&amp;I e a geração de conhecimentos e soluções para políticas públicas."
+Público-alvo: "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas. A equipe executora deve ser exclusiva e composta por no mínimo 7 pesquisadores doutores, além do coordenador, com representação da Instituição Executora, outras IES/P capixabas, IES/P de fora do estado ou do País, e um pesquisador vinculado a órgão ou instituição pública estadual." → "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Espírito Santo. O coordenador deve liderar uma equipe que inclua pesquisadores doutores da Instituição Executora, de outras IES/P capixabas, de IES/P de fora do estado ou do País, e um pesquisador de órgão ou instituição pública estadual relacionada à temática da proposta."</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>O edital visa apoiar financeiramente a criação e o fortalecimento de redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos no Espírito Santo. O objetivo é consolidar grupos de referência em áreas do conhecimento e setores estratégicos, promovendo ações coletivas de PD&amp;I e a geração de conhecimentos e soluções para políticas públicas.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Espírito Santo. O coordenador deve liderar uma equipe que inclua pesquisadores doutores da Instituição Executora, de outras IES/P capixabas, de IES/P de fora do estado ou do País, e um pesquisador de órgão ou instituição pública estadual relacionada à temática da proposta.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 12.000.000,00</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>R$ 1.200.000,00</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-07 a 2026-09-21: Envio da proposta e documentos (até as 17h59, via SigFapes)
+2026-09-10: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
+2026-10-01: Prazo para recorrer (habilitação) (Até 5 dias úteis após a divulgação do resultado preliminar)
+2026-11-17: Prazo para recorrer (análise de mérito) (Até 5 dias úteis após a divulgação do resultado preliminar)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>O coordenador é responsável pelo conteúdo e integridade da proposta, bem como por obter as licenças e autorizações necessárias para a execução do projeto. A Fapes pode solicitar documentos complementares para corrigir falhas formais, desde que não impliquem alteração substancial da proposta. A Fapes não se responsabiliza por propostas não recebidas devido a inadimplências do proponente, problemas técnicos de rede (exceto os causados pelas plataformas da Fapes) ou encerramento do prazo. Atendimento especializado para acessibilidade pode ser solicitado até 10 dias antes do prazo final de envio das propostas.</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_21-2026_-_Redes_de_PDI_em_Setores_Estratégicos-1.pdf</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>pesquisa/EDITAL_FAPES_No_21_2026_-_REDES_DE_PESQUISA,_DESENVOLVIMENTO_E_INOVAÇÃO_EM_SETORES_ESTRATÉGICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisa</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>EDITAL FAPES Nº 24/2026 - PRIMEIROS PROJETOS DE PESQUISA - ESPÍRITO SANTO (PPP-ES)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr"/>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>O Edital Fapes n° 24/2026 (PPP-ES) tem como objetivo apoiar o primeiro projeto de pesquisa científica de pesquisadores doutores em início de carreira. Ele visa promover o acesso a recursos para o desenvolvimento de seus primeiros projetos, fortalecer a infraestrutura de pesquisa e apoiar a formação e consolidação de novos grupos de pesquisa no Estado do Espírito Santo. Os projetos devem estar vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, localizadas no Espírito Santo, e contemplar as 8 grandes áreas do conhecimento do CNPq, com duração de até 24 meses.</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores doutores em início de carreira, com título obtido a partir de 28/08/2018, que possuam vínculo estatutário ou celetista por tempo indeterminado com uma Instituição de Ensino Superior e/ou de Pesquisa (IES/P) pública ou privada localizada no Espírito Santo, residam no Espírito Santo ou em município limítrofe, e que não tenham atuado como coordenador de projetos de pesquisa, extensão ou inovação no âmbito da Fapes ou do CNPq (com exceções específicas).</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>R$ 4.000.000,00</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>R$ 180.000,00</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>2026-09-28: Prazo para envio de dúvidas a respeito do edital (até as 17h59)
 2026-08-29 a 2026-09-30: Envio da proposta e documentos (até as 17h59, via SigFapes)
@@ -782,76 +858,70 @@
 2026-12-10: Envio de documentos para contratação (O coordenador receberá informações com prazo e documentação necessária via SigFapes.)</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
         <is>
           <t>Projetos aprovados terão duração máxima de 24 meses e devem estar enquadrados em uma das 8 grandes áreas do conhecimento do CNPq. A Fapes reserva-se o direito de alterar as datas e prazos do cronograma por necessidade administrativa ou decisão institucional. É fundamental que o coordenador mantenha seus dados cadastrais atualizados no sistema SigFapes para garantir o recebimento das comunicações oficiais. A proposta aprovada não poderá ser alterada no momento da contratação, e a ausência da documentação ética e legal exigida impedirá a contratação do projeto.</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20Fapes%2024-2026%20PPP-ES.pdf</t>
         </is>
       </c>
-      <c r="N5" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>pesquisa/EDITAL_FAPES_No_24_2026_-_PRIMEIROS_PROJETOS_DE_PESQUISA_-_ESPÍRITO_SANTO_(PPP-ES).pdf</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 17/2026 - PRÊMIO FAPES DE CIÊNCIA, TECNOLOGIA, INOVAÇÃO E JORNALISMO – EDIÇÃO 2026</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 16/09/2026</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (Até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 28/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação. Ele busca valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, e ampliar a divulgação e popularização da ciência no estado." → "O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Os objetivos específicos incluem valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, ampliar a divulgação da ciência e fortalecer a visibilidade institucional da Fundação."
-Público-alvo: "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes (executados entre 01/01/2019 e 31/12/2025), e profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou a programas/projetos fomentados." → "Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também se destina a profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação."
-Valor por proposta: "R$ 12.000,00" → "R$ 12.000,00 (1º lugar); R$ 8.000,00 (menção honrosa)"</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>O Prêmio Fapes tem como objetivo reconhecer e premiar projetos de destaque e trajetórias profissionais nas áreas de pesquisa, extensão e inovação, bem como premiar matérias jornalísticas sobre a Fapes ou programas e projetos fomentados pela Fundação. Os objetivos específicos incluem valorizar a relevância e o impacto da pesquisa, extensão e inovação para o desenvolvimento do Espírito Santo, reconhecer a excelência de profissionais apoiados pela Fapes, ampliar a divulgação da ciência e fortalecer a visibilidade institucional da Fundação.</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores, extensionistas e empreendedores vinculados a projetos contratados pela Fapes, executados a partir de 01/01/2019 e concluídos até 31/12/2025. Também se destina a profissionais de jornalismo residentes no Espírito Santo, autores de matérias relacionadas à Fapes ou aos programas e projetos fomentados pela Fundação.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>R$ 308.000,00</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>R$ 12.000,00 (1º lugar); R$ 8.000,00 (menção honrosa)</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>2026-06-22 a 2026-08-06: Envio das inscrições – Categorias Projetos e Destaque (Até 17h59)
 2026-06-22 a 2026-09-28: Envio das inscrições – Categoria Jornalismo (Até 17h59. A matéria deve ter sido veiculada entre 01/09/2025 a 28/09/2026 e disponibilizada no canal oficial do veículo de comunicação.)
@@ -859,70 +929,70 @@
 2026-11-03 a 2026-11-09: Votação popular – Categoria Jornalismo (Votação entre as 3 matérias mais bem classificadas em cada subcategoria.)</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
         <is>
           <t>Esta edição do Prêmio Fapes homenageia a Professora Jurema José de Oliveira. Os valores das premiações possuem natureza bruta e estão sujeitos à incidência do Imposto de Renda Retido na Fonte – IRRF. A premiação possui caráter exclusivamente honorífico, meritório e eventual, não configurando contraprestação por serviços prestados, vínculo empregatício, relação de trabalho, bolsa de pesquisa ou remuneração continuada. É permitida apenas uma inscrição por pessoa neste edital, sendo a última enviada considerada válida em caso de múltiplas submissões. A Fapes garante condições de acessibilidade às pessoas com deficiência durante o processo de inscrição. O participante autoriza o uso de seu nome, imagem, voz e demais informações para fins institucionais e de divulgação do prêmio, sem remuneração. O tratamento dos dados pessoais seguirá a Lei Federal nº 13.709/2018 (LGPD).</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_17.2026_Prêmio_Fapes_Edição_2026_Professora_Jurema_José_de_Oliveira.pdf</t>
         </is>
       </c>
-      <c r="N6" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_17_2026_-_PRÊMIO_FAPES_DE_CIÊNCIA,_TECNOLOGIA,_INOVAÇÃO_E_JORNALISMO_–_EDIÇÃO_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr"/>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>R$ 200.000,00</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
 2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
@@ -931,70 +1001,70 @@
 2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
         <is>
           <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
         </is>
       </c>
-      <c r="N7" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Difusão do Conhecimento</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
         <is>
           <t>Removido (nao mais aberto)</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
 2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
@@ -1015,70 +1085,70 @@
 2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Extensão</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 01/2026 – TCC EMPREENDEDOR INOVADOR</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>2026-09-02 a 2026-10-27: Período de submissão das propostas (Segunda Chamada) (Até as 17h59)</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>O edital visa incentivar o desenvolvimento de Trabalhos de Conclusão de Curso (TCC) com foco em inovação, empreendedorismo e aplicabilidade prática. Serão concedidas Bolsas de Apoio a Trabalho de Conclusão de Curso (BTCC) para propostas que apresentem soluções inovadoras e empreendedoras, com impacto econômico, social e/ou ambiental no Espírito Santo, alinhadas aos ODS da ONU (especialmente 4, 8, 9, 10 e 17) e ao Plano ES 500 Anos.</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Podem submeter propostas professores orientadores com vínculo estatutário ou celetista por tempo indeterminado a IES reconhecidas pelo MEC e localizadas no Espírito Santo, que não estejam afastados da IES, estejam adimplentes com a FAPES, residam no ES ou municípios limítrofes, e possuam currículo Lattes atualizado. Cada proponente deve submeter entre 3 e 5 propostas, cada uma vinculada a um único aluno. Se os alunos orientados estiverem vinculados a outra IES, o proponente deve apresentar declaração de autorização de ambas as IES. Os alunos orientados devem ser estudantes regulares de graduação em IES localizadas no Espírito Santo, com desempenho acadêmico igual ou superior a 7.0, adimplentes com a FAPES, com o proponente como professor orientador durante todo o período da bolsa, residência no ES ou municípios limítrofes, e cadastrados no Sigfapes. As IES devem ser públicas ou privadas, localizadas no ES, e prestar anuência às propostas.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>R$ 1.600.000,00</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>R$ 11.000,00</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>editais.extensao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>2026-02-02 a 2026-03-30: Período de submissão das propostas (Primeira Chamada) (Até as 17h59)
 ?: Prazo para interposição de recursos administrativos (Primeira Chamada) (5 (cinco) dias úteis a partir da publicação do resultado de seleção)
@@ -1091,70 +1161,70 @@
 ?: Prazo de contratação (Terceira Chamada) (Até 5 (cinco) dias úteis da publicação do resultado homologado)</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
         <is>
           <t>O edital aceita todos os formatos de TCC definido pelas DCNs, como monografia, dissertação, projeto experimental, relatório técnico ou científico, artigo, plano de negócios e outros. As propostas concorrerão com as demais de suas respectivas microrregiões. Serão apoiados no máximo 20 projetos de TCC por microrregião na primeira chamada, e até 10 projetos de TCC por microrregião nas segunda e terceira chamadas. Recursos financeiros remanescentes serão destinados a projetos em ampla concorrência por ordem decrescente de nota. Propostas submetidas a mais de uma microrregião serão desclassificadas. Propostas com Nota Final (NF) inferior a 70 pontos serão desclassificadas. Em caso de empate na NF, serão utilizados os critérios de avaliação 1, 2, 3, 4 e 5, nesta ordem, para desempate. Persistindo o empate, será selecionada a proposta submetida primeiro. Não é permitido o acúmulo de bolsas FAPES com outras bolsas, exceto as do Programa Nossa Bolsa, Programa Universidade para Todos (Prouni) e Bolsas de Extensão (Ext-E e Ext-F). O prazo de execução dos projetos será de um semestre letivo, acrescido de até 3 meses apenas para apresentação da Declaração ou Ata de Defesa do TCC. O valor da bolsa BTCC e do Auxílio para orientação de TCC são fixados na Tabela de Valores de Bolsas e Auxílios da Fapes (https://fapes.es.gov.br/valores-de-bolsas-e-auxilios) na data de publicação deste edital. A modalidade de concessão da bolsa é por cooperação financeira não reembolsável. O orientador receberá até dois auxílios para orientação de TCC: o primeiro após a contratação e o segundo quando pelo menos um aluno orientado apresentar a Ata de Defesa do TCC. Cada proposta de TCC aprovada será contemplada com bolsa BTCC com duração mínima de 2 meses e máxima de 4 meses, não prorrogáveis.</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/EDITAL_FAPES_Nº_01.2026_TCC_EMPREENDEDOR_INOVADOR-2.pdf</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>extensao/EDITAL_FAPES_No_01_2026_–_TCC_EMPREENDEDOR_INOVADOR.pdf</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES Nº 08/2026 - NOVA ECONOMIA CAPIXABA 2026</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>O objetivo principal do Edital 08/2026 (Nova Economia Capixaba) é promover um significativo aumento de competitividade dos setores econômicos capixabas no cenário nacional por meio de projetos de inovação a partir de demandas das empresas, em colaboração com ICT ou IES capixabas, públicas ou privadas. O apoio aos projetos de inovação se dará por meio de um modelo de coinvestimento tripartite entre a FAPES, a empresa proponente e a ICT/IES, com recursos não reembolsáveis da FAPES, contrapartida econômica da ICT/IES e contrapartida financeira da empresa.</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Empresas com sede administrativa ou filial no Espírito Santo, individualmente ou em associação com outras empresas capixabas, e Cooperativas de Trabalho (produção e serviço) somente como empresa coexecutora. As empresas proponentes e coexecutoras devem ter receita bruta operacional superior a R$ 360.000,00 nos dois últimos exercícios fiscais.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>R$ 40.000.000,00</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>Entre R$ 500.000,00 e R$ 3.000.000,00</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br, suporte@fapes.es.gov.br, sucon@fapes.es.gov.br, contacorrente@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>2026-08-01: Submissão das propostas no SIGFAPES (Fluxo contínuo)
 2026-10-04 a 2026-10-10: Prazo de submissão dos recursos administrativos (Habilitação) (05 (cinco) dias úteis a partir da publicação do resultado preliminar.)
@@ -1164,157 +1234,89 @@
 ?: Início da vigência dos Termo de Outorga (A partir do primeiro dia do mês subsequente à assinatura do Termo de Outorga.)</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>O edital foi alterado em 01/08/2026. Cooperativas de Trabalho (produção e serviço) podem participar como empresas coexecutoras. As regras de elegibilidade para empresas que participaram de editais FAPES anteriores (Tecnova III, Nova Economia Capixaba, Apoio aos Clusters de Inovação Capixaba) foram atualizadas, permitindo a submissão se o projeto, coordenador e equipe forem distintos. Novas regras para ressubmissão de propostas após inabilitação ou reprovação pelo Comitê de Conformidade foram adicionadas. O Termo de Outorga (ANEXO VIII) inclui agora cláusulas específicas sobre material permanente e sigilo.</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_08-2026_-_Nova_Economia_Capixaba_-_2_Edição_-_Lançamento.pdf</t>
         </is>
       </c>
-      <c r="N10" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_No_08_2026_-_NOVA_ECONOMIA_CAPIXABA_2026.pdf</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Inovação</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>EDITAL FAPES N° 23/2026 - APOIO ÀS INCUBADORAS DO ESPÍRITO SANTO</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr"/>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Apoiar incubadoras públicas ou privadas sem fins lucrativos, localizadas no Espírito Santo, com o objetivo de fornecer apoio logístico, gerencial e/ou tecnológico a empreendedores e empresas que desenvolvam produtos, serviços ou modelos de negócio inovadores. O edital visa ampliar, aperfeiçoar e consolidar as atividades de pré-incubação, incubação e pós-incubação, estimulando a capacitação de novos empreendedores, a sustentabilidade econômica das empresas incubadas e a promoção da inovação no Espírito Santo.</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Incubadoras, sem fins lucrativos, sediadas no Espírito Santo.</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>R$ 4.500.000,00</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I12" s="2" t="inlineStr">
         <is>
           <t>R$ 252.000,00</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
         <is>
           <t>duvidas.inovacao@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>2026-08-25 a 2026-09-24: Envio da proposta e documentos (até as 17h59, via SigFapes)
 ?: Prazo para recorrer (Até 5 dias úteis após a divulgação do resultado preliminar de habilitação e análise de mérito)
 2026-11-04: Contratação dos projetos selecionados (A partir desta data)</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
         <is>
           <t>Os valores por proposta variam conforme o nível de maturidade da incubadora: Nível Avançado (R$ 252.000,00), Nível Intermediário (R$ 192.000,00) e Nível Básico (R$ 132.000,00). Propostas com nota final inferior a 60 pontos serão desclassificadas. A classificação por nível de maturidade é baseada nas seguintes pontuações: Nível Avançado (86 a 100 pontos), Nível Intermediário (76 a 85 pontos) e Nível Básico (60 a 75 pontos). Os recursos financeiros remanescentes serão redirecionados para propostas suplentes nos níveis de maturidade I, II e III, nesta ordem, respeitando a classificação. O projeto terá prazo de vigência de 24 meses, sem prorrogação. Mínimo de 20% do valor total solicitado deve ser destinado a bolsas. Parte dos recursos de custeio deve ser destinada à associação à Anprotec. Serão permitidas exclusivamente bolsas na modalidade BPIG, níveis II a X, por no máximo 24 meses.</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_23-2026_Apoio%20a%20Incubadoras_(Versão%20Final).pdf</t>
         </is>
       </c>
-      <c r="N11" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>inovacao/EDITAL_FAPES_N°_23_2026_-_APOIO_ÀS_INCUBADORAS_DO_ESPÍRITO_SANTO.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Chamadas Internacionais</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CHAMADA CONFAP CDTI 2026</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>€ 75.000,00</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1326,7 +1328,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
+          <t>CHAMADA CONFAP CDTI 2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1336,53 +1338,53 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
+          <t>Este edital visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha, abrangendo qualquer setor de atividade. O financiamento é destinado a profissionais vinculados a universidades, centros de pesquisa ou empresas capixabas que realizem atividades de pesquisa, desenvolvimento e inovação tecnológica. É necessário que as propostas integrem uma parceria conjunta com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
+          <t>Pesquisadores principais ou coordenadores de projetos, brasileiros ou estrangeiros com visto permanente, que residam no estado do Espírito Santo e possuam vínculo ativo com universidades, centros de pesquisa ou empresas localizadas no Espírito Santo. Os proponentes devem estar adimplentes com a FAPES na data limite de submissão e não ter projetos anteriores CONFAP CDTI vigentes no momento da contratação. É mandatório que as propostas sejam conjuntas com uma empresa espanhola.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>R$ 300.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>R$ 150.000,00</t>
+          <t>€ 75.000,00</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, brasil@cdti.es, carlos.quintana@cdti.es, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+          <t>2026-10-08: Submissão de propostas (até as 23:59 (horário de Brasília) na plataforma do CONFAP (https://sistema.confap.org.br). Formulários devem ser preenchidos em língua inglesa.)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
+          <t>A Chamada CONFAP &amp; CDTI visa apoiar projetos colaborativos em pesquisa e inovação tecnológica entre o Brasil e a Espanha. As propostas devem ser submetidas na plataforma do CONFAP, preenchidas em inglês, e incluir o Formulário de Projeto de Cooperação Tecnológica Internacional e o Acordo de Consórcio. Cada proponente pode submeter apenas uma proposta. A duração dos projetos varia de 12 a 36 meses. O apoio financeiro da FAPES destina-se a despesas de capital e custeio, excluindo bolsas, conforme Resolução nº 309/2022. A submissão à FAPES ocorre somente após a aprovação da proposta pelo CDTI. O orçamento total mínimo do projeto deve ser de 250.000,00 Euros, com o apoio da FAPES compondo no mínimo 30% da contrapartida.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes_Chamada%20Internacional_CDTI.2026.pdf</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_CDTI_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1394,7 +1396,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA ERC-CONFAP 2026</t>
+          <t>CHAMADA CONFAP &amp; WBI - BÉLGICA 2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1402,52 +1404,55 @@
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
+        </is>
+      </c>
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+          <t>Apoiar projetos conjuntos de Pesquisa e Inovação, promovendo o intercâmbio científico entre grupos de pesquisa do Espírito Santo e da região da Valônia-Bruxelas, na Bélgica, em áreas como inovação em saúde, energia sustentável, gestão ambiental e aeronáutica. Os projetos devem ser inovadores, agregar valor e resultar em publicações científicas conjuntas.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+          <t>Pesquisadores brasileiros com doutorado, vinculados a Instituições de Ensino Superior e/ou Pesquisa (IES/P) localizadas no estado do Espírito Santo, residentes no estado, que atuem como pesquisador principal ou coordenador do projeto, e que participem de propostas conjuntas com pesquisadores da Valônia-Bruxelas, Bélgica.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>US$ 18.000,00</t>
+          <t>R$ 300.000,00</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>US$ 6.000,00</t>
+          <t>R$ 150.000,00</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+          <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
-2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+          <t>2026-09-30: Submissão de propostas (Até as 23h59min (horário de Brasília) via https://sistema.confap.org.br)</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+          <t>O prazo de vigência máximo para cada projeto é de 24 meses. O apoio financeiro da Fapes destina-se exclusivamente a despesas de mobilidade, como passagens aéreas internacionais e auxílio para missões técnico-científicas na Bélgica, excluindo bolsas. Os valores dos auxílios são definidos na Resolução FAPES/CCAF 361/2026. Cada proponente pode submeter apenas uma proposta; em caso de múltiplas submissões, a última será considerada. As propostas devem usar o modelo do Anexo I e ser submetidas em ambas as plataformas (CONFAP). A execução dos projetos não poderá exceder a vigência dos acordos entre a Fapes e as instituições fomentadoras.</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20WBI%20-2026.pdf</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+          <t>chamadas_internacionais/CHAMADA_CONFAP_&amp;_WBI_-_BÉLGICA_2026.pdf</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1464,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>CHAMADA HORIZON EUROPE</t>
+          <t>CHAMADA ERC-CONFAP 2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1471,96 +1476,161 @@
       <c r="E15" s="2" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
+          <t>Apoiar a mobilidade de pesquisadores do estado do Espírito Santo para integrar equipes de pesquisa na Europa, em projetos financiados pelo Conselho Europeu de Pesquisa (ERC). O edital visa promover colaborações de pesquisa e fortalecer a internacionalização da ciência, tecnologia e inovação desenvolvida no Espírito Santo, permitindo missões científicas de 6 a 12 meses ou visitas curtas.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Pesquisadores doutores, principais ou coordenadores de projeto, ativos em pesquisa, vinculados a Instituições de Ensino Superior ou Pesquisa (IES/P) localizadas no estado do Espírito Santo. Devem possuir currículo Lattes atualizado, ser residentes no ES, e ser brasileiros ou estrangeiros com visto permanente, além de estar adimplentes junto à FAPES.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 18.000,00</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>US$ 6.000,00</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>internacional.confap@gmail.com, global@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-10: Submissão de propostas (CONFAP) (Via plataforma CONFAP, preenchendo informações de interesse e dados pessoais.)
+2026-08-10: Submissão de propostas (FAPES) (Via SigFapes, para verificação de elegibilidade e documentação exigida, conforme Instrução de Serviços nº 082/2025 e Item 4, alínea B.)</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Este edital da FAPES apresenta diretrizes específicas para a Chamada ERC – CONFAP 2026. Os resultados serão publicados na página do CONFAP: http://www.confap.org.br/. Os pesquisadores selecionados continuarão a receber seus salários e/ou bolsas de acordo com os termos e condições institucionais. O apoio da FAPES destina-se a custeio de passagens aéreas, seguro viagem e mobilidade.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Chamada-ERC-CONFAP-2026.pdf</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>chamadas_internacionais/CHAMADA_ERC-CONFAP_2026.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Chamadas Internacionais</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>CHAMADA HORIZON EUROPE</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
           <t>Este edital da FAPES visa apoiar a participação de pesquisadores do estado do Espírito Santo, na condição de co-PI (co-Principal Investigator), em projetos de pesquisa e inovação executados por consórcios de parceiros europeus e associados no âmbito do Programa Horizonte Europa. As diretrizes orientam exclusivamente a submissão de propostas na categoria “C - Projetos Colaborativos (Pilar II)”, que se refere a projetos de pesquisa e inovação em grande escala para desenvolver soluções para desafios globais.</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores proponentes do estado do Espírito Santo, na condição de co-PI, vinculados a instituições de pesquisa ou acadêmicas, para participação em consórcios de projetos colaborativos da categoria 'C - Projetos Colaborativos (Pilar II)' do Horizonte Europa.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>€ 25.000,00 por ano de projeto</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>parcerias@fapes.es.gov.br, internacional.confap@confap.org.br</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>?: Consulta de Elegibilidade à FAPES (Pesquisadores devem consultar a FAPES sobre sua elegibilidade antes de iniciar a preparação da proposta, enviando informações como CV em inglês, nome e instituição do coordenador da proposta do Horizonte Europa, título da proposta, orçamento estimado, duração do projeto e descrição resumida.)
 ?: Submissão da Proposta à FAPES (A FAPES receberá propostas associadas às chamadas do Horizonte Europa a qualquer momento. A proposta deve incluir cópia da proposta em inglês submetida ao Horizonte Europa, seguir diretrizes da FAPES e indicar detalhes da proposta vinculada.)
 ?: Assinatura do Termo de Outorga FAPES (Disponível somente após a submissão do Acordo de Subvenção com o qual a UE concede o apoio financeiro ao consórcio. O cofinanciamento por parte da Fapes somente poderá ser contratado até o término da vigência do Arranjo Administrativo Horizonte Europa 2021–2027.)</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>Os parceiros do Brasil não podem ser coordenadores das propostas submetidas ao Horizonte Europa, pois não são automaticamente elegíveis para receber financiamento da UE. Portanto, eles não podem ser responsáveis pela gestão administrativa e financeira geral do projeto; eles só podem participar como parceiros (ou co-PIs). A referência da chamada é o título (Programa/Tópico) e o número da chamada. Os recursos financeiros aplicados pela Fapes para financiamento de projetos no contexto do Horizonte Europa serão oriundos do Fundo Estadual de Ciência e Tecnologia do Espírito Santo - Funcitec, fonte 0159, recursos vinculados ao Tesouro do Estado. Outros recursos financeiros, decorrentes de parcerias futuras ou de disponibilidade da Fapes e/ou do Funcitec, poderão ser aplicados na suplementação de propostas aprovadas no âmbito do Horizonte Europa 2021-2027. O número máximo de propostas a serem apoiadas no âmbito destas Diretrizes é de até 2 (DOIS) projetos por ano do Horizonte Europa 2021-2027. Os recursos financeiros aprovados pela Fundação poderão abranger despesas com passagens e diárias, observando suas respectivas regulamentações disponíveis na Resolução CCAF nº 309/2022.</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Diretrizes%20Fapes%20Horizon%20Europe%202021-2027-1.pdf</t>
         </is>
       </c>
-      <c r="N15" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_HORIZON_EUROPE.pdf</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Chamadas Internacionais</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>CHAMADA DA PARCERIA DE MATÉRIAS-PRIMAS PARA A TRANSIÇÃO VERDE E DIGITAL (RAMP)</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C17" s="2" t="inlineStr">
         <is>
           <t>Sem alteracoes</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr"/>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Este edital visa financiar projetos de pesquisa e/ou inovação em toda a cadeia de valor de matérias-primas. Os projetos devem focar em melhorar o acesso a matérias-primas, promover práticas de economia circular, alcançar a sustentabilidade e minimizar custos sociais e ambientais, agregando valor e contribuindo para o desenvolvimento industrial.</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Pesquisadores e instituições vinculadas a organizações de ensino superior e centros de pesquisa públicos no Espírito Santo. Outras entidades devem verificar a elegibilidade diretamente com a FAPES.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>EUR 100.000,00</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
         <is>
           <t>internacional.confap@gmail.com, global4@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>2026-09-22: Prazo final para submissão de pré-propostas (até as 15:00 CEST)
 2026-10-06 a 2026-10-15: Período para interposição de recursos (Elegibilidade Etapa 1) (Janela de 10 dias para recursos)
@@ -1572,17 +1642,17 @@
 2027-06-01 a 2027-09-30: Negociações de contrato nacional/regional e início dos projetos (previsto)</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
         <is>
           <t>O edital se aplica a todas as matérias-primas não combustíveis e não alimentares, com foco em matérias-primas críticas/estratégicas, mas sem ser essencial. Cada proposta multilateral deve envolver no mínimo três parceiros de três países diferentes, solicitando financiamento de um dos financiadores participantes. Financiadores de pelo menos dois desses países devem ser elegíveis para receber cofinanciamento da Comissão Europeia. O escopo temático abrange a cadeia de suprimentos primária e secundária, design e produção, e uso e reutilização de produtos e componentes. Para a FAPES, todas as faixas de TRL (1-9) são elegíveis. Recomenda-se que os candidatos verifiquem se as FAPs em seus respectivos estados definiram um valor mínimo ou máximo de financiamento por projeto e se exigem submissão de proposta através da plataforma da FAP dentro do prazo de chamada.</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital%20-%20Chamada%20RAMP%202026.pdf</t>
         </is>
       </c>
-      <c r="N16" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>chamadas_internacionais/CHAMADA_DA_PARCERIA_DE_MATÉRIAS-PRIMAS_PARA_A_TRANSIÇÃO_VERDE_E_DIGITAL_(RAMP).pdf</t>
         </is>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-18 11:50
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -29,17 +29,12 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -54,15 +49,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -606,7 +598,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>2026-07-31 a 2026-09-17: Prazo para impugnação do edital (Até 5 dias úteis anteriores ao encerramento do prazo de envio das propostas.)</t>
+          <t>2026-09-24: Submissão das propostas (Até as 17h59, via Sistema de Informação e Gestão de Projetos da Fapes.)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -737,9 +729,9 @@
           <t>EDITAL FAPES Nº 21/2026 - REDES DE PESQUISA, DESENVOLVIMENTO E INOVAÇÃO EM SETORES ESTRATÉGICOS</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>Atualizado - e-mail enviado em 17/09/2026</t>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -747,12 +739,7 @@
           <t>2026-08-07 a 2026-09-21: Envio da proposta e documentos (até as 17h59, via SigFapes)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Objetivo: "O edital Redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos visa apoiar financeiramente a criação e o fortalecimento de redes que promovam ações coletivas de PD&amp;I. Seu objetivo geral é selecionar projetos para criar e fortalecer redes estruturantes de PD&amp;I em setores estratégicos e de interesse do Espírito Santo, bem como consolidar grupos de referência em áreas do conhecimento e setores estratégicos do estado." → "O edital visa apoiar financeiramente a criação e o fortalecimento de redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos no Espírito Santo. O objetivo é consolidar grupos de referência em áreas do conhecimento e setores estratégicos, promovendo ações coletivas de PD&amp;I e a geração de conhecimentos e soluções para políticas públicas."
-Público-alvo: "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Estado do Espírito Santo, que atuem como coordenadores de propostas. A equipe executora deve ser exclusiva e composta por no mínimo 7 pesquisadores doutores, além do coordenador, com representação da Instituição Executora, outras IES/P capixabas, IES/P de fora do estado ou do País, e um pesquisador vinculado a órgão ou instituição pública estadual." → "Pesquisadores doutores vinculados a Instituições de Ensino Superior e/ou de Pesquisa (IES/P) públicas ou privadas, sediadas no Espírito Santo. O coordenador deve liderar uma equipe que inclua pesquisadores doutores da Instituição Executora, de outras IES/P capixabas, de IES/P de fora do estado ou do País, e um pesquisador de órgão ou instituição pública estadual relacionada à temática da proposta."</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>O edital visa apoiar financeiramente a criação e o fortalecimento de redes de Pesquisa, Desenvolvimento e Inovação (PD&amp;I) em Setores Estratégicos no Espírito Santo. O objetivo é consolidar grupos de referência em áreas do conhecimento e setores estratégicos, promovendo ações coletivas de PD&amp;I e a geração de conhecimentos e soluções para políticas públicas.</t>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-19 11:12
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -940,38 +940,38 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
+          <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
+          <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>R$ 3.000.000,00</t>
+          <t>R$ 800.000,00</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>R$ 200.000,00</t>
+          <t>US$ 1.500,00</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -980,78 +980,6 @@
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
-2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
-2026-10-23 a 2026-10-29: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
-2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
-2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 800.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
 2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
@@ -1072,19 +1000,91 @@
 2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 200.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
+2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
+2026-10-23 a 2026-10-29: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
+2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
+        </is>
+      </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
+          <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-20 11:31
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -940,46 +940,118 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Removido (nao mais aberto)</t>
+          <t>Sem alteracoes</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
+          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
+          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>R$ 200.000,00</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
+2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
+2026-10-23 a 2026-10-29: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
+2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Removido (nao mais aberto)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
           <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>R$ 800.000,00</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>US$ 1.500,00</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
         <is>
           <t>editais.duvidas@fapes.es.gov.br</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
 2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
@@ -1000,91 +1072,19 @@
 2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
         <is>
           <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Sem alteracoes</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 3.000.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 200.000,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
-2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
-2026-10-23 a 2026-10-29: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
-2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
-2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(editais): atualizacao automatica 2026-09-21 13:49
</commit_message>
<xml_diff>
--- a/editais_fapes/_extracao.xlsx
+++ b/editais_fapes/_extracao.xlsx
@@ -940,38 +940,38 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
+          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Sem alteracoes</t>
+          <t>Removido (nao mais aberto)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
+          <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
+          <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
+          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>R$ 3.000.000,00</t>
+          <t>R$ 800.000,00</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>R$ 200.000,00</t>
+          <t>US$ 1.500,00</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -980,78 +980,6 @@
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
-2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
-2026-10-23 a 2026-10-29: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
-2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
-2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Difusão do Conhecimento</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>EDITAL FAPES Nº 28/2025 - PUBLICAÇÃO DE ARTIGOS TÉCNICO-CIENTÍFICOS</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Removido (nao mais aberto)</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-06 a 2026-10-26: Submissão de propostas - 4ª Chamada (Até as 17h59.)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>O edital visa incentivar a publicação científica e tecnológica no Espírito Santo, concedendo auxílio financeiro para artigos técnico-científicos resultantes de pesquisas desenvolvidas em Instituições de Ensino e/ou Pesquisa no estado. Os objetivos específicos incluem valorizar a produção técnico-científica de pesquisadores e alunos capixabas, ampliar a visibilidade das produções e fomentar a cultura de publicação científica.</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Pesquisador ou aluno em atividade de pesquisa ou desenvolvimento inovador em Instituição de Ensino e/ou Pesquisa (IES/P) localizada no estado do Espírito Santo.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>R$ 800.000,00</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>US$ 1.500,00</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>editais.duvidas@fapes.es.gov.br</t>
-        </is>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>2025-12-22 a 2026-02-25: Submissão de propostas - 1ª Chamada (Até as 17h59.)
 2026-02-18: Prazo para impugnação do edital (Até 5 dias úteis antes do encerramento da submissão da 1ª chamada.)
@@ -1072,19 +1000,91 @@
 2026-12-31 a 2027-01-29: Informar dados bancários - 4ª Chamada (Prazo de até 30 dias a partir da publicação da contratação no DIO-ES.)</t>
         </is>
       </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Difusão do Conhecimento</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>EDITAL FAPES Nº 25/2026 - CIÊNCIA ABERTA CAPIXABA</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Sem alteracoes</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08: Prazo para envio de dúvidas (Até as 17h59)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Apoiar projetos voltados à organização, disponibilização, disseminação e aplicação de dados, informações e evidências científicas de interesse público. O edital busca ampliar o acesso ao conhecimento científico produzido no Espírito Santo, fortalecer sua integração a redes e sistemas de informação nacionais e internacionais e promover sua comunicação para diferentes segmentos da sociedade, contribuindo para enfrentar o desafio da desinformação. O foco é construir uma infraestrutura pública de dados e conhecimento científico.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Profissionais/pesquisadores doutores e vinculados a Instituições de Ensino Superior/ou de Pesquisa (IES/P) sediadas no Estado do Espírito Santo.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 3.000.000,00</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>R$ 200.000,00</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>editais.duvidas@fapes.es.gov.br</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 a 2026-10-15: Envio da proposta e documentos (Até as 17h59, via SigFapes)
+2026-10-08: Prazo para envio de dúvidas (Até as 17h59)
+2026-10-23 a 2026-10-29: Prazo para recorrer (habilitação) (5 dias úteis após a divulgação do resultado preliminar da habilitação)
+2026-11-11 a 2026-11-17: Prazo para recorrer (análise de mérito) (5 dias úteis após a divulgação do resultado preliminar de análise de mérito)
+2026-12-10: Início da contratação dos projetos selecionados (A partir desta data)</t>
+        </is>
+      </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>O edital prevê 4 chamadas para submissão de propostas. O proponente poderá ser contratado para no máximo 2 propostas, desde que submetidas em chamadas distintas. No entanto, o item 7.10 do edital original afirma que 'Cada coordenador pode apresentar apenas uma proposta a este edital. Caso enviem mais de uma proposta, será considerada apenas a última enviada.', o que pode gerar contradição com a possibilidade de contratação de até 2 propostas em chamadas distintas. O prazo máximo para execução de cada projeto é de 12 meses. A produção será analisada com base na classificação Qualis (2021-2024) ou no percentil Scopus/Web of Science.</t>
+          <t>O prazo de execução do projeto é de 24 meses. O orçamento deve prever 24 meses de bolsa na modalidade de Iniciação Científica e Tecnológica (ICT) da Fapes. As propostas devem se enquadrar em uma das linhas temáticas: Saúde e Saúde Pública; Sustentabilidade Socioambiental, Descarbonização e Clima; Biodiversidade e Recursos Naturais; Cidades e Territórios Sustentáveis e Resilientes; Agricultura, Produção de Alimentos e Segurança Alimentar. O foco do edital é construir uma infraestrutura pública de dados e conhecimento científico, não financiar pesquisas. Cada coordenador pode apresentar apenas uma proposta. A equipe executora deve ser composta pelo coordenador e, no mínimo, mais 2 (dois) pesquisadores doutores de IES/P de fora do Estado. Documentos de aprovação ética e legal podem estar em análise na submissão, mas devem estar aprovados para a contratação.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_28_2025_Publicação_de_Artigos_Técnico-Científicos.pdf</t>
+          <t>https://fapes.es.gov.br/Media/fapes/Editais/Edital_Fapes_25-2026_Ciência_Aberta_Capixaba.pdf</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>difusao_do_conhecimento/EDITAL_FAPES_No_28_2025_-_PUBLICAÇÃO_DE_ARTIGOS_TÉCNICO-CIENTÍFICOS.pdf</t>
+          <t>difusao_do_conhecimento/EDITAL_FAPES_No_25_2026_-_CIÊNCIA_ABERTA_CAPIXABA.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>